<commit_message>
wip: para volver a la firma
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -28,13 +28,13 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>01-00 LLAVE</t>
+    <t>01-00 IPAD</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
   </si>
   <si>
-    <t>14-FEBRERO-2025</t>
+    <t>17-FEBRERO-2025</t>
   </si>
   <si>
     <t>De acuerdo con la “AS-DV-002. Uso de recursos informáticos”, me comprometo a utilizar el hardware y/o software que se me asigno, exclusivamente para actividades relacionadas con los negocios de la empresa, así como a cuidarlo y mantenerlo en buen estado</t>
@@ -46,12 +46,12 @@
     <t>Equipo ACR</t>
   </si>
   <si>
+    <t>X</t>
+  </si>
+  <si>
     <t>Equipo Externo</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>CANT</t>
   </si>
   <si>
@@ -70,16 +70,16 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>AFADSFASF</t>
-  </si>
-  <si>
-    <t>AFDSFASF</t>
-  </si>
-  <si>
-    <t>ADFSASDF</t>
-  </si>
-  <si>
-    <t>PRUEBA</t>
+    <t>SADFASDf</t>
+  </si>
+  <si>
+    <t>ASDFAS</t>
+  </si>
+  <si>
+    <t>ASDFADS</t>
+  </si>
+  <si>
+    <t>ASDF</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1287,14 +1287,14 @@
       <c r="B19" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="13"/>
+      <c r="C19" s="13" t="s">
+        <v>9</v>
+      </c>
       <c r="F19" s="33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G19" s="33"/>
-      <c r="H19" s="13" t="s">
-        <v>10</v>
-      </c>
+      <c r="H19" s="13"/>
       <c r="L19" s="22"/>
     </row>
     <row r="20" spans="1:14" customHeight="1" ht="7.5"/>

</xml_diff>

<commit_message>
wip: trabajando para pantalla emerjente en create_mante.php
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -28,13 +28,13 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>01-00 MOUSE</t>
+    <t>01-00 PC-COMPLETA</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
   </si>
   <si>
-    <t>01-FEBRERO-2025</t>
+    <t>18-FEBRERO-2025</t>
   </si>
   <si>
     <t>De acuerdo con la “AS-DV-002. Uso de recursos informáticos”, me comprometo a utilizar el hardware y/o software que se me asigno, exclusivamente para actividades relacionadas con los negocios de la empresa, así como a cuidarlo y mantenerlo en buen estado</t>
@@ -46,12 +46,12 @@
     <t>Equipo ACR</t>
   </si>
   <si>
+    <t>X</t>
+  </si>
+  <si>
     <t>Equipo Externo</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>CANT</t>
   </si>
   <si>
@@ -70,10 +70,13 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>ASDF</t>
-  </si>
-  <si>
-    <t>ASSDF</t>
+    <t>QE</t>
+  </si>
+  <si>
+    <t>QEWR</t>
+  </si>
+  <si>
+    <t>QWER</t>
   </si>
   <si>
     <t>N/A</t>
@@ -102,19 +105,16 @@
     <t>Jose Arturo Moreno Aguilar</t>
   </si>
   <si>
-    <t>Mario Javier Romero Mendoza</t>
-  </si>
-  <si>
     <t>Abel de Jesús Mora Flores</t>
   </si>
   <si>
     <t>Julio Castillo Valerdi</t>
   </si>
   <si>
-    <t>Auliira Contable</t>
-  </si>
-  <si>
-    <t>Soporte 2</t>
+    <t>Garantias</t>
+  </si>
+  <si>
+    <t>Soporte 1</t>
   </si>
   <si>
     <t>Coordinador soporte</t>
@@ -1276,14 +1276,14 @@
       <c r="B19" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="25"/>
+      <c r="C19" s="25" t="s">
+        <v>9</v>
+      </c>
       <c r="F19" s="34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G19" s="34"/>
-      <c r="H19" s="25" t="s">
-        <v>10</v>
-      </c>
+      <c r="H19" s="25"/>
       <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:14" customHeight="1" ht="7.5"/>
@@ -1317,7 +1317,7 @@
     <row r="22" spans="1:14" customHeight="1" ht="26.25">
       <c r="A22" s="2"/>
       <c r="B22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>17</v>
@@ -1326,19 +1326,19 @@
       <c r="E22" s="41"/>
       <c r="F22" s="42"/>
       <c r="G22" s="37" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
       <c r="J22" s="39"/>
       <c r="K22" s="22" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="L22" s="23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M22" s="22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
@@ -1426,7 +1426,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1469,7 +1469,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1486,7 +1486,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1499,10 +1499,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L33" s="51" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1562,7 +1562,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1749,7 +1749,7 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>

</xml_diff>

<commit_message>
se hizo media query para adaptar imagen a resolucion de panalla
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="37">
   <si>
     <t>Automóviles y Camiones Rivera, S.A. de C.V.</t>
   </si>
@@ -28,7 +28,7 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>01-00 LLAVE</t>
+    <t>01-00 PC-COMPLETA</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
@@ -70,16 +70,10 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>DADSFAS</t>
-  </si>
-  <si>
-    <t>FASDF</t>
-  </si>
-  <si>
-    <t>ASDFA</t>
-  </si>
-  <si>
-    <t>ASDF</t>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>ENSAMBLE</t>
   </si>
   <si>
     <t>N/A</t>
@@ -112,9 +106,6 @@
   </si>
   <si>
     <t>Julio Castillo Valerdi</t>
-  </si>
-  <si>
-    <t>Auxliar</t>
   </si>
   <si>
     <t>Soporte 1</t>
@@ -1335,13 +1326,13 @@
       <c r="I22" s="38"/>
       <c r="J22" s="39"/>
       <c r="K22" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" s="23">
+        <v>12354889</v>
+      </c>
+      <c r="M22" s="22" t="s">
         <v>19</v>
-      </c>
-      <c r="L22" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="M22" s="22" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
@@ -1429,7 +1420,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1472,7 +1463,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1489,7 +1480,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1502,10 +1493,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L33" s="51" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1565,7 +1556,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1752,23 +1743,23 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>
       <c r="E56" s="47"/>
       <c r="F56" s="45" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G56" s="46"/>
       <c r="H56" s="47"/>
       <c r="I56" s="20"/>
       <c r="J56" s="45" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K56" s="47"/>
       <c r="L56" s="45" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M56" s="47"/>
     </row>
@@ -1788,23 +1779,23 @@
     </row>
     <row r="58" spans="1:14" customHeight="1" ht="13.5">
       <c r="B58" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="49"/>
       <c r="E58" s="50"/>
       <c r="F58" s="48" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G58" s="49"/>
       <c r="H58" s="50"/>
       <c r="I58" s="20"/>
       <c r="J58" s="48" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="K58" s="50"/>
       <c r="L58" s="48" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="M58" s="50"/>
     </row>
@@ -1910,29 +1901,29 @@
     </row>
     <row r="66" spans="1:14" customHeight="1" ht="12.75">
       <c r="B66" s="64" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C66" s="65"/>
       <c r="D66" s="65"/>
       <c r="E66" s="66"/>
       <c r="F66" s="59" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G66" s="67"/>
       <c r="H66" s="60"/>
       <c r="J66" s="67" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K66" s="60"/>
       <c r="L66" s="59" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M66" s="60"/>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="L71" s="17"/>
     </row>

</xml_diff>

<commit_message>
wip: se sube directorio aun falta trabajar boton de agregar
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="37">
   <si>
     <t>Automóviles y Camiones Rivera, S.A. de C.V.</t>
   </si>
@@ -28,13 +28,13 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>02-00 OTRO</t>
+    <t>01-00 PC-COMPLETA</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
   </si>
   <si>
-    <t>26-FEBRERO-2025</t>
+    <t>10-MARZO-2025</t>
   </si>
   <si>
     <t>De acuerdo con la “AS-DV-002. Uso de recursos informáticos”, me comprometo a utilizar el hardware y/o software que se me asigno, exclusivamente para actividades relacionadas con los negocios de la empresa, así como a cuidarlo y mantenerlo en buen estado</t>
@@ -70,16 +70,10 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>ADSAD</t>
-  </si>
-  <si>
-    <t>ASDASD</t>
-  </si>
-  <si>
-    <t>ASDAS</t>
-  </si>
-  <si>
-    <t>ASDASD PERRO</t>
+    <t>AFSDF</t>
+  </si>
+  <si>
+    <t>ASDF</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1317,7 +1311,7 @@
     <row r="22" spans="1:14" customHeight="1" ht="26.25">
       <c r="A22" s="2"/>
       <c r="B22" s="21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>17</v>
@@ -1332,13 +1326,13 @@
       <c r="I22" s="38"/>
       <c r="J22" s="39"/>
       <c r="K22" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="M22" s="22" t="s">
         <v>19</v>
-      </c>
-      <c r="L22" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="M22" s="22" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
@@ -1426,7 +1420,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1469,7 +1463,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1486,7 +1480,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1499,10 +1493,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L33" s="51" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1562,7 +1556,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1749,23 +1743,23 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>
       <c r="E56" s="47"/>
       <c r="F56" s="45" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G56" s="46"/>
       <c r="H56" s="47"/>
       <c r="I56" s="20"/>
       <c r="J56" s="45" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K56" s="47"/>
       <c r="L56" s="45" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M56" s="47"/>
     </row>
@@ -1785,23 +1779,23 @@
     </row>
     <row r="58" spans="1:14" customHeight="1" ht="13.5">
       <c r="B58" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="49"/>
       <c r="E58" s="50"/>
       <c r="F58" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G58" s="49"/>
       <c r="H58" s="50"/>
       <c r="I58" s="20"/>
       <c r="J58" s="48" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K58" s="50"/>
       <c r="L58" s="48" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M58" s="50"/>
     </row>
@@ -1907,29 +1901,29 @@
     </row>
     <row r="66" spans="1:14" customHeight="1" ht="12.75">
       <c r="B66" s="64" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C66" s="65"/>
       <c r="D66" s="65"/>
       <c r="E66" s="66"/>
       <c r="F66" s="59" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G66" s="67"/>
       <c r="H66" s="60"/>
       <c r="J66" s="67" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K66" s="60"/>
       <c r="L66" s="59" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M66" s="60"/>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="L71" s="17"/>
     </row>

</xml_diff>

<commit_message>
se corrigen errores de funciones
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -28,13 +28,13 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>01-00 PC-COMPLETA</t>
+    <t>02-00 OTRO</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
   </si>
   <si>
-    <t>10-MARZO-2025</t>
+    <t>12-MARZO-2025</t>
   </si>
   <si>
     <t>De acuerdo con la “AS-DV-002. Uso de recursos informáticos”, me comprometo a utilizar el hardware y/o software que se me asigno, exclusivamente para actividades relacionadas con los negocios de la empresa, así como a cuidarlo y mantenerlo en buen estado</t>
@@ -70,10 +70,7 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>AFSDF</t>
-  </si>
-  <si>
-    <t>ASDF</t>
+    <t>TT</t>
   </si>
   <si>
     <t>N/A</t>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>Julio Castillo Valerdi</t>
+  </si>
+  <si>
+    <t>Tt</t>
   </si>
   <si>
     <t>Soporte 1</t>
@@ -1311,7 +1311,7 @@
     <row r="22" spans="1:14" customHeight="1" ht="26.25">
       <c r="A22" s="2"/>
       <c r="B22" s="21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>17</v>
@@ -1320,19 +1320,19 @@
       <c r="E22" s="41"/>
       <c r="F22" s="42"/>
       <c r="G22" s="37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H22" s="38"/>
       <c r="I22" s="38"/>
       <c r="J22" s="39"/>
       <c r="K22" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="L22" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="M22" s="22" t="s">
         <v>18</v>
-      </c>
-      <c r="L22" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="M22" s="22" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
@@ -1420,7 +1420,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1463,7 +1463,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1480,7 +1480,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1493,10 +1493,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="L33" s="51" t="s">
         <v>23</v>
-      </c>
-      <c r="L33" s="51" t="s">
-        <v>24</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1556,7 +1556,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1743,23 +1743,23 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>
       <c r="E56" s="47"/>
       <c r="F56" s="45" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G56" s="46"/>
       <c r="H56" s="47"/>
       <c r="I56" s="20"/>
       <c r="J56" s="45" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K56" s="47"/>
       <c r="L56" s="45" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M56" s="47"/>
     </row>
@@ -1779,7 +1779,7 @@
     </row>
     <row r="58" spans="1:14" customHeight="1" ht="13.5">
       <c r="B58" s="48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="49"/>

</xml_diff>

<commit_message>
se restablecio tamaño canvas por temas de formato
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="38">
   <si>
     <t>Automóviles y Camiones Rivera, S.A. de C.V.</t>
   </si>
@@ -28,13 +28,13 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>04-00 PC-COMPLETA</t>
+    <t>05-00 PC-COMPLETA</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
   </si>
   <si>
-    <t>23-ABRIL-2025</t>
+    <t>24-ABRIL-2025</t>
   </si>
   <si>
     <t>De acuerdo con la “AS-DV-002. Uso de recursos informáticos”, me comprometo a utilizar el hardware y/o software que se me asigno, exclusivamente para actividades relacionadas con los negocios de la empresa, así como a cuidarlo y mantenerlo en buen estado</t>
@@ -76,28 +76,10 @@
     <t>ENSAMBLE</t>
   </si>
   <si>
+    <t>123456789ABCEFGHIJKL7</t>
+  </si>
+  <si>
     <t>N/A</t>
-  </si>
-  <si>
-    <t>MONITOR</t>
-  </si>
-  <si>
-    <t>LENOVO</t>
-  </si>
-  <si>
-    <t>SJSJ4</t>
-  </si>
-  <si>
-    <t>COMBO T/M</t>
-  </si>
-  <si>
-    <t>LOGITECH</t>
-  </si>
-  <si>
-    <t>K200</t>
-  </si>
-  <si>
-    <t>12392929N</t>
   </si>
   <si>
     <t>CARACTERISTICAS DEL SOFTWARE</t>
@@ -1349,66 +1331,42 @@
       <c r="K22" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="L22" s="23">
-        <v>1299790</v>
+      <c r="L22" s="23" t="s">
+        <v>19</v>
       </c>
       <c r="M22" s="22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="21">
-        <v>1</v>
-      </c>
-      <c r="C23" s="40" t="s">
-        <v>20</v>
-      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="40"/>
       <c r="D23" s="41"/>
       <c r="E23" s="41"/>
       <c r="F23" s="42"/>
-      <c r="G23" s="37" t="s">
-        <v>21</v>
-      </c>
+      <c r="G23" s="37"/>
       <c r="H23" s="38"/>
       <c r="I23" s="38"/>
       <c r="J23" s="39"/>
-      <c r="K23" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="L23" s="24">
-        <v>123456789</v>
-      </c>
-      <c r="M23" s="22" t="s">
-        <v>19</v>
-      </c>
+      <c r="K23" s="22"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="22"/>
     </row>
     <row r="24" spans="1:14" customHeight="1" ht="26.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="21">
-        <v>1</v>
-      </c>
-      <c r="C24" s="40" t="s">
-        <v>23</v>
-      </c>
+      <c r="B24" s="21"/>
+      <c r="C24" s="40"/>
       <c r="D24" s="41"/>
       <c r="E24" s="41"/>
       <c r="F24" s="42"/>
-      <c r="G24" s="37" t="s">
-        <v>24</v>
-      </c>
+      <c r="G24" s="37"/>
       <c r="H24" s="38"/>
       <c r="I24" s="38"/>
       <c r="J24" s="39"/>
-      <c r="K24" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="L24" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="M24" s="22" t="s">
-        <v>19</v>
-      </c>
+      <c r="K24" s="22"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="22"/>
     </row>
     <row r="25" spans="1:14" customHeight="1" ht="26.25">
       <c r="B25" s="21"/>
@@ -1465,7 +1423,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1508,7 +1466,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1525,7 +1483,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1538,10 +1496,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="L33" s="51" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1601,7 +1559,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1788,23 +1746,23 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>
       <c r="E56" s="47"/>
       <c r="F56" s="45" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G56" s="46"/>
       <c r="H56" s="47"/>
       <c r="I56" s="20"/>
       <c r="J56" s="45" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="K56" s="47"/>
       <c r="L56" s="45" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="M56" s="47"/>
     </row>
@@ -1824,23 +1782,23 @@
     </row>
     <row r="58" spans="1:14" customHeight="1" ht="13.5">
       <c r="B58" s="48" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="49"/>
       <c r="E58" s="50"/>
       <c r="F58" s="48" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G58" s="49"/>
       <c r="H58" s="50"/>
       <c r="I58" s="20"/>
       <c r="J58" s="48" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K58" s="50"/>
       <c r="L58" s="48" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="M58" s="50"/>
     </row>
@@ -1946,29 +1904,29 @@
     </row>
     <row r="66" spans="1:14" customHeight="1" ht="12.75">
       <c r="B66" s="64" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C66" s="65"/>
       <c r="D66" s="65"/>
       <c r="E66" s="66"/>
       <c r="F66" s="59" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G66" s="67"/>
       <c r="H66" s="60"/>
       <c r="J66" s="67" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="K66" s="60"/>
       <c r="L66" s="59" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M66" s="60"/>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="L71" s="17"/>
     </row>

</xml_diff>

<commit_message>
Wip:exportar a excel el directorio
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
+++ b/imagenes_guardadas/archivo_modificado_RESGUARDO.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="39">
   <si>
     <t>Automóviles y Camiones Rivera, S.A. de C.V.</t>
   </si>
@@ -28,7 +28,7 @@
     <t>No. de Resguardo:</t>
   </si>
   <si>
-    <t>05-00 PC-COMPLETA</t>
+    <t>06-00 PC-COMPLETA</t>
   </si>
   <si>
     <t>Fecha de resguardo:</t>
@@ -46,12 +46,12 @@
     <t>Equipo ACR</t>
   </si>
   <si>
+    <t>X</t>
+  </si>
+  <si>
     <t>Equipo Externo</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>CANT</t>
   </si>
   <si>
@@ -70,13 +70,16 @@
     <t>Inv. Físico</t>
   </si>
   <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>ENSAMBLE</t>
-  </si>
-  <si>
-    <t>123456789ABCEFGHIJKL7</t>
+    <t>GGG</t>
+  </si>
+  <si>
+    <t>YG</t>
+  </si>
+  <si>
+    <t>GGY</t>
+  </si>
+  <si>
+    <t>TGG</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1273,14 +1276,14 @@
       <c r="B19" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="25"/>
+      <c r="C19" s="25" t="s">
+        <v>9</v>
+      </c>
       <c r="F19" s="34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G19" s="34"/>
-      <c r="H19" s="25" t="s">
-        <v>10</v>
-      </c>
+      <c r="H19" s="25"/>
       <c r="L19" s="18"/>
     </row>
     <row r="20" spans="1:14" customHeight="1" ht="7.5"/>
@@ -1329,13 +1332,13 @@
       <c r="I22" s="38"/>
       <c r="J22" s="39"/>
       <c r="K22" s="22" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L22" s="23" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M22" s="22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:14" customHeight="1" ht="26.25">
@@ -1423,7 +1426,7 @@
     </row>
     <row r="29" spans="1:14" customHeight="1" ht="7.5" hidden="true">
       <c r="B29" s="30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
@@ -1466,7 +1469,7 @@
     <row r="32" spans="1:14" customHeight="1" ht="14.45">
       <c r="A32" s="2"/>
       <c r="B32" s="35" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="35"/>
@@ -1483,7 +1486,7 @@
     <row r="33" spans="1:14" customHeight="1" ht="14.45">
       <c r="A33" s="2"/>
       <c r="B33" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>12</v>
@@ -1496,10 +1499,10 @@
       <c r="I33" s="36"/>
       <c r="J33" s="36"/>
       <c r="K33" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L33" s="51" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M33" s="52"/>
     </row>
@@ -1559,7 +1562,7 @@
     <row r="41" spans="1:14" customHeight="1" ht="6"/>
     <row r="42" spans="1:14" customHeight="1" ht="13.5">
       <c r="B42" s="43" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C42" s="44"/>
       <c r="D42" s="44"/>
@@ -1746,23 +1749,23 @@
     </row>
     <row r="56" spans="1:14" customHeight="1" ht="13.5">
       <c r="B56" s="45" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C56" s="46"/>
       <c r="D56" s="46"/>
       <c r="E56" s="47"/>
       <c r="F56" s="45" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G56" s="46"/>
       <c r="H56" s="47"/>
       <c r="I56" s="20"/>
       <c r="J56" s="45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K56" s="47"/>
       <c r="L56" s="45" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M56" s="47"/>
     </row>
@@ -1782,23 +1785,23 @@
     </row>
     <row r="58" spans="1:14" customHeight="1" ht="13.5">
       <c r="B58" s="48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="49"/>
       <c r="E58" s="50"/>
       <c r="F58" s="48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G58" s="49"/>
       <c r="H58" s="50"/>
       <c r="I58" s="20"/>
       <c r="J58" s="48" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K58" s="50"/>
       <c r="L58" s="48" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M58" s="50"/>
     </row>
@@ -1904,29 +1907,29 @@
     </row>
     <row r="66" spans="1:14" customHeight="1" ht="12.75">
       <c r="B66" s="64" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C66" s="65"/>
       <c r="D66" s="65"/>
       <c r="E66" s="66"/>
       <c r="F66" s="59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G66" s="67"/>
       <c r="H66" s="60"/>
       <c r="J66" s="67" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K66" s="60"/>
       <c r="L66" s="59" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M66" s="60"/>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L71" s="17"/>
     </row>

</xml_diff>